<commit_message>
finishing making the model robust, dispatch, and have an export electricity option that connects to reducing the CO2 emission)
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,28 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Paper - Nuclear DACSS\Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0746133-CDC5-4EBC-9614-3C32DA8DB4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C9CA35D-B5AD-4A9D-86AE-61024D73B2BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="11295" firstSheet="12" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31665" yWindow="135" windowWidth="17295" windowHeight="15510" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="country" sheetId="1" r:id="rId1"/>
-    <sheet name="energy_duty" sheetId="2" r:id="rId2"/>
-    <sheet name="env_condition" sheetId="3" r:id="rId3"/>
-    <sheet name="co2_tax" sheetId="4" r:id="rId4"/>
-    <sheet name="co2_storage_capacity" sheetId="5" r:id="rId5"/>
-    <sheet name="capex" sheetId="6" r:id="rId6"/>
-    <sheet name="gdp" sheetId="7" r:id="rId7"/>
-    <sheet name="nuclear_allowed" sheetId="8" r:id="rId8"/>
-    <sheet name="ccs_readiness" sheetId="9" r:id="rId9"/>
-    <sheet name="nuclear_readiness" sheetId="10" r:id="rId10"/>
-    <sheet name="nuclear_perception" sheetId="11" r:id="rId11"/>
-    <sheet name="resource_reserve" sheetId="12" r:id="rId12"/>
-    <sheet name="ccs_included" sheetId="13" r:id="rId13"/>
-    <sheet name="non-NPT" sheetId="14" r:id="rId14"/>
+    <sheet name="energy_duty_adjusted" sheetId="15" r:id="rId2"/>
+    <sheet name="energy_duty" sheetId="2" r:id="rId3"/>
+    <sheet name="env_condition" sheetId="3" r:id="rId4"/>
+    <sheet name="co2_tax" sheetId="4" r:id="rId5"/>
+    <sheet name="co2_storage_capacity" sheetId="5" r:id="rId6"/>
+    <sheet name="capex" sheetId="6" r:id="rId7"/>
+    <sheet name="gdp" sheetId="7" r:id="rId8"/>
+    <sheet name="nuclear_allowed" sheetId="8" r:id="rId9"/>
+    <sheet name="ccs_readiness" sheetId="9" r:id="rId10"/>
+    <sheet name="nuclear_readiness" sheetId="10" r:id="rId11"/>
+    <sheet name="nuclear_perception" sheetId="11" r:id="rId12"/>
+    <sheet name="resource_reserve" sheetId="12" r:id="rId13"/>
+    <sheet name="ccs_included" sheetId="13" r:id="rId14"/>
+    <sheet name="non-NPT" sheetId="14" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">nuclear_perception!$A$1:$C$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">nuclear_perception!$A$1:$C$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1096,6 +1097,804 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:B193"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="1"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="1"/>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="1"/>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="1"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="1"/>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="1"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="1"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="1"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="1"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="1"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="1"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="1"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="1"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="1"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="1"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="1"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="1"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="1"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="1"/>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="1"/>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="1"/>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="1"/>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1"/>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="1"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="1"/>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="1"/>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="1"/>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="1"/>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="1"/>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="1"/>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="1"/>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" s="1"/>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" s="1"/>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" s="1"/>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" s="1"/>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" s="1"/>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" s="1"/>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" s="1"/>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" s="1"/>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" s="1"/>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" s="1"/>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" s="1"/>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" s="1"/>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" s="1"/>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" s="1"/>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" s="1"/>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" s="1"/>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" s="1"/>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" s="1"/>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" s="1"/>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" s="1"/>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" s="1"/>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" s="1"/>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" s="1"/>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" s="1"/>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" s="1"/>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" s="1"/>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" s="1"/>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" s="1"/>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" s="1"/>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" s="1"/>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" s="1"/>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" s="1"/>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" s="1"/>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" s="1"/>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" s="1"/>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" s="1"/>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" s="1"/>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" s="1"/>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" s="1"/>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112" s="1"/>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113" s="1"/>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" s="1"/>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" s="1"/>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" s="1"/>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" s="1"/>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" s="1"/>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" s="1"/>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" s="1"/>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" s="1"/>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" s="1"/>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" s="1"/>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" s="1"/>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" s="1"/>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" s="1"/>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" s="1"/>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A128" s="1"/>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A129" s="1"/>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A130" s="1"/>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131" s="1"/>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132" s="1"/>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133" s="1"/>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A134" s="1"/>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135" s="1"/>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A136" s="1"/>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A137" s="1"/>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A138" s="1"/>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A139" s="1"/>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A140" s="1"/>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A141" s="1"/>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A142" s="1"/>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A143" s="1"/>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A144" s="1"/>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A145" s="1"/>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A146" s="1"/>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A147" s="1"/>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A148" s="1"/>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A149" s="1"/>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A150" s="1"/>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A151" s="1"/>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A152" s="1"/>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A153" s="1"/>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A154" s="1"/>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A155" s="1"/>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A156" s="1"/>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A157" s="1"/>
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A158" s="1"/>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A159" s="1"/>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A160" s="1"/>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A161" s="1"/>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A162" s="1"/>
+    </row>
+    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A163" s="1"/>
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A164" s="1"/>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A165" s="1"/>
+    </row>
+    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A166" s="1"/>
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A167" s="1"/>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A168" s="1"/>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A169" s="1"/>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A170" s="1"/>
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A171" s="1"/>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A172" s="1"/>
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A173" s="1"/>
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A174" s="1"/>
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A175" s="1"/>
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A176" s="1"/>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A177" s="1"/>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A178" s="1"/>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A179" s="1"/>
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A180" s="1"/>
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A181" s="1"/>
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A182" s="1"/>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A183" s="1"/>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A184" s="1"/>
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A185" s="1"/>
+    </row>
+    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A186" s="1"/>
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A187" s="1"/>
+    </row>
+    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A188" s="1"/>
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A189" s="1"/>
+    </row>
+    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A190" s="1"/>
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A191" s="1"/>
+    </row>
+    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A192" s="1"/>
+    </row>
+    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A193" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:B193"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1894,7 +2693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:C193"/>
   <sheetFormatPr defaultColWidth="23.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2969,7 +3768,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:C193"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4195,7 +4994,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:A176"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4789,7 +5588,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4815,6 +5614,1245 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4263980-EA7E-45E7-B5BB-DC7057FF7490}">
+  <dimension ref="A1:R22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B1">
+        <v>0</v>
+      </c>
+      <c r="C1">
+        <v>2.5</v>
+      </c>
+      <c r="D1">
+        <v>5</v>
+      </c>
+      <c r="E1">
+        <v>7.5</v>
+      </c>
+      <c r="F1">
+        <v>10</v>
+      </c>
+      <c r="G1">
+        <v>12.5</v>
+      </c>
+      <c r="H1">
+        <v>15</v>
+      </c>
+      <c r="I1">
+        <v>17.5</v>
+      </c>
+      <c r="J1">
+        <v>20</v>
+      </c>
+      <c r="K1">
+        <v>22.5</v>
+      </c>
+      <c r="L1">
+        <v>25</v>
+      </c>
+      <c r="M1">
+        <v>27.5</v>
+      </c>
+      <c r="N1">
+        <v>30</v>
+      </c>
+      <c r="O1">
+        <v>32.5</v>
+      </c>
+      <c r="P1">
+        <v>35</v>
+      </c>
+      <c r="Q1">
+        <v>37.5</v>
+      </c>
+      <c r="R1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>6.7991541551655654</v>
+      </c>
+      <c r="C2">
+        <v>6.7571619229923741</v>
+      </c>
+      <c r="D2">
+        <v>6.7413631225864385</v>
+      </c>
+      <c r="E2">
+        <v>6.7255643221805039</v>
+      </c>
+      <c r="F2">
+        <v>6.754224005649335</v>
+      </c>
+      <c r="G2">
+        <v>6.782883689118167</v>
+      </c>
+      <c r="H2">
+        <v>6.5729125353360676</v>
+      </c>
+      <c r="I2">
+        <v>6.3629413815539708</v>
+      </c>
+      <c r="J2">
+        <v>6.2457544540647909</v>
+      </c>
+      <c r="K2">
+        <v>6.1285675265756083</v>
+      </c>
+      <c r="L2">
+        <v>5.9738472060916861</v>
+      </c>
+      <c r="M2">
+        <v>5.819126885607762</v>
+      </c>
+      <c r="N2">
+        <v>5.7732594005582758</v>
+      </c>
+      <c r="O2">
+        <v>5.7273919155087887</v>
+      </c>
+      <c r="P2">
+        <v>5.6647962888530161</v>
+      </c>
+      <c r="Q2">
+        <v>5.6022006621972418</v>
+      </c>
+      <c r="R2">
+        <v>5.4483437296671955</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>7.7462807476477851</v>
+      </c>
+      <c r="C3">
+        <v>7.4911016412809683</v>
+      </c>
+      <c r="D3">
+        <v>7.3578161259018664</v>
+      </c>
+      <c r="E3">
+        <v>7.2245306105227645</v>
+      </c>
+      <c r="F3">
+        <v>7.0228935487954169</v>
+      </c>
+      <c r="G3">
+        <v>6.8212564870680676</v>
+      </c>
+      <c r="H3">
+        <v>6.5000042192312648</v>
+      </c>
+      <c r="I3">
+        <v>6.1787519513944611</v>
+      </c>
+      <c r="J3">
+        <v>6.2744441162820159</v>
+      </c>
+      <c r="K3">
+        <v>6.3701362811695725</v>
+      </c>
+      <c r="L3">
+        <v>6.1958398379815245</v>
+      </c>
+      <c r="M3">
+        <v>6.0215433947934764</v>
+      </c>
+      <c r="N3">
+        <v>6.0488840133327768</v>
+      </c>
+      <c r="O3">
+        <v>6.0762246318720772</v>
+      </c>
+      <c r="P3">
+        <v>6.0078730855238218</v>
+      </c>
+      <c r="Q3">
+        <v>5.9395215391755665</v>
+      </c>
+      <c r="R3">
+        <v>5.604501317002903</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>7.5805282477532696</v>
+      </c>
+      <c r="C4">
+        <v>7.4637610227416671</v>
+      </c>
+      <c r="D4">
+        <v>7.2706679043078424</v>
+      </c>
+      <c r="E4">
+        <v>7.0775747858740177</v>
+      </c>
+      <c r="F4">
+        <v>6.9955529302561121</v>
+      </c>
+      <c r="G4">
+        <v>6.9135310746382057</v>
+      </c>
+      <c r="H4">
+        <v>6.6606303531496609</v>
+      </c>
+      <c r="I4">
+        <v>6.4077296316611179</v>
+      </c>
+      <c r="J4">
+        <v>6.4213999409307689</v>
+      </c>
+      <c r="K4">
+        <v>6.4350702502004182</v>
+      </c>
+      <c r="L4">
+        <v>6.2556474410362481</v>
+      </c>
+      <c r="M4">
+        <v>6.0762246318720772</v>
+      </c>
+      <c r="N4">
+        <v>6.0283785494283002</v>
+      </c>
+      <c r="O4">
+        <v>5.9805324669845215</v>
+      </c>
+      <c r="P4">
+        <v>5.9002194000253194</v>
+      </c>
+      <c r="Q4">
+        <v>5.81990633306612</v>
+      </c>
+      <c r="R4">
+        <v>5.5886990904542957</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>15</v>
+      </c>
+      <c r="B5">
+        <v>7.4147757478587533</v>
+      </c>
+      <c r="C5">
+        <v>7.4364204042023676</v>
+      </c>
+      <c r="D5">
+        <v>7.1835196827138184</v>
+      </c>
+      <c r="E5">
+        <v>6.93061896122527</v>
+      </c>
+      <c r="F5">
+        <v>6.9682123117168064</v>
+      </c>
+      <c r="G5">
+        <v>7.0058056622083447</v>
+      </c>
+      <c r="H5">
+        <v>6.8212564870680596</v>
+      </c>
+      <c r="I5">
+        <v>6.6367073119277755</v>
+      </c>
+      <c r="J5">
+        <v>6.5683557655795202</v>
+      </c>
+      <c r="K5">
+        <v>6.5000042192312648</v>
+      </c>
+      <c r="L5">
+        <v>6.3154550440909718</v>
+      </c>
+      <c r="M5">
+        <v>6.1309058689506779</v>
+      </c>
+      <c r="N5">
+        <v>6.0078730855238218</v>
+      </c>
+      <c r="O5">
+        <v>5.8848403020969657</v>
+      </c>
+      <c r="P5">
+        <v>5.7925657145268197</v>
+      </c>
+      <c r="Q5">
+        <v>5.7002911269566727</v>
+      </c>
+      <c r="R5">
+        <v>5.5728968639056866</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>20</v>
+      </c>
+      <c r="B6">
+        <v>7.4663811653516792</v>
+      </c>
+      <c r="C6">
+        <v>7.4500907134720133</v>
+      </c>
+      <c r="D6">
+        <v>7.2433272857685367</v>
+      </c>
+      <c r="E6">
+        <v>7.0365638580650627</v>
+      </c>
+      <c r="F6">
+        <v>7.0416902240411794</v>
+      </c>
+      <c r="G6">
+        <v>7.0468165900172988</v>
+      </c>
+      <c r="H6">
+        <v>6.8605586262183067</v>
+      </c>
+      <c r="I6">
+        <v>6.674300662419312</v>
+      </c>
+      <c r="J6">
+        <v>6.4812075439854926</v>
+      </c>
+      <c r="K6">
+        <v>6.2881144255516705</v>
+      </c>
+      <c r="L6">
+        <v>6.1616640648073968</v>
+      </c>
+      <c r="M6">
+        <v>6.0352137040631222</v>
+      </c>
+      <c r="N6">
+        <v>5.9668621577148668</v>
+      </c>
+      <c r="O6">
+        <v>5.8985106113666115</v>
+      </c>
+      <c r="P6">
+        <v>5.7925657145268152</v>
+      </c>
+      <c r="Q6">
+        <v>5.6866208176870181</v>
+      </c>
+      <c r="R6">
+        <v>5.4864484319528453</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>25</v>
+      </c>
+      <c r="B7">
+        <v>7.5179865828446042</v>
+      </c>
+      <c r="C7">
+        <v>7.4637610227416582</v>
+      </c>
+      <c r="D7">
+        <v>7.3031348888232568</v>
+      </c>
+      <c r="E7">
+        <v>7.1425087549048545</v>
+      </c>
+      <c r="F7">
+        <v>7.1151681363655541</v>
+      </c>
+      <c r="G7">
+        <v>7.0878275178262538</v>
+      </c>
+      <c r="H7">
+        <v>6.8998607653685511</v>
+      </c>
+      <c r="I7">
+        <v>6.7118940129108493</v>
+      </c>
+      <c r="J7">
+        <v>6.3940593223914632</v>
+      </c>
+      <c r="K7">
+        <v>6.0762246318720772</v>
+      </c>
+      <c r="L7">
+        <v>6.0078730855238218</v>
+      </c>
+      <c r="M7">
+        <v>5.9395215391755665</v>
+      </c>
+      <c r="N7">
+        <v>5.9258512299059118</v>
+      </c>
+      <c r="O7">
+        <v>5.9121809206362581</v>
+      </c>
+      <c r="P7">
+        <v>5.7925657145268108</v>
+      </c>
+      <c r="Q7">
+        <v>5.6729505084173635</v>
+      </c>
+      <c r="R7">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>30</v>
+      </c>
+      <c r="B8">
+        <v>7.6127673937808602</v>
+      </c>
+      <c r="C8">
+        <v>7.5013543732332053</v>
+      </c>
+      <c r="D8">
+        <v>7.3612337032192805</v>
+      </c>
+      <c r="E8">
+        <v>7.2211130332053557</v>
+      </c>
+      <c r="F8">
+        <v>7.1220032910003859</v>
+      </c>
+      <c r="G8">
+        <v>7.0228935487954169</v>
+      </c>
+      <c r="H8">
+        <v>6.8622674148770146</v>
+      </c>
+      <c r="I8">
+        <v>6.7016412809586123</v>
+      </c>
+      <c r="J8">
+        <v>6.4948778532551419</v>
+      </c>
+      <c r="K8">
+        <v>6.2881144255516705</v>
+      </c>
+      <c r="L8">
+        <v>6.1479937555377457</v>
+      </c>
+      <c r="M8">
+        <v>6.0078730855238218</v>
+      </c>
+      <c r="N8">
+        <v>5.9412303278342709</v>
+      </c>
+      <c r="O8">
+        <v>5.8745875701447208</v>
+      </c>
+      <c r="P8">
+        <v>5.7874393485506914</v>
+      </c>
+      <c r="Q8">
+        <v>5.7002911269566638</v>
+      </c>
+      <c r="R8">
+        <v>5.4387162687529749</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>35</v>
+      </c>
+      <c r="B9">
+        <v>7.7075482047171153</v>
+      </c>
+      <c r="C9">
+        <v>7.5389477237247497</v>
+      </c>
+      <c r="D9">
+        <v>7.4193325176153033</v>
+      </c>
+      <c r="E9">
+        <v>7.299717311505856</v>
+      </c>
+      <c r="F9">
+        <v>7.1288384456352176</v>
+      </c>
+      <c r="G9">
+        <v>6.9579595797645792</v>
+      </c>
+      <c r="H9">
+        <v>6.8246740643854773</v>
+      </c>
+      <c r="I9">
+        <v>6.6913885490063763</v>
+      </c>
+      <c r="J9">
+        <v>6.5956963841188205</v>
+      </c>
+      <c r="K9">
+        <v>6.5000042192312648</v>
+      </c>
+      <c r="L9">
+        <v>6.2881144255516705</v>
+      </c>
+      <c r="M9">
+        <v>6.0762246318720772</v>
+      </c>
+      <c r="N9">
+        <v>5.9566094257626307</v>
+      </c>
+      <c r="O9">
+        <v>5.8369942196531834</v>
+      </c>
+      <c r="P9">
+        <v>5.7823129825745738</v>
+      </c>
+      <c r="Q9">
+        <v>5.7276317454959642</v>
+      </c>
+      <c r="R9">
+        <v>5.4774325375059503</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>40</v>
+      </c>
+      <c r="B10">
+        <v>7.8595164760980589</v>
+      </c>
+      <c r="C10">
+        <v>7.6995738576431432</v>
+      </c>
+      <c r="D10">
+        <v>7.5406565123834497</v>
+      </c>
+      <c r="E10">
+        <v>7.3817391671237571</v>
+      </c>
+      <c r="F10">
+        <v>7.2091515125944143</v>
+      </c>
+      <c r="G10">
+        <v>7.0365638580650707</v>
+      </c>
+      <c r="H10">
+        <v>6.9101134973207969</v>
+      </c>
+      <c r="I10">
+        <v>6.7836631365765232</v>
+      </c>
+      <c r="J10">
+        <v>6.5888612294839923</v>
+      </c>
+      <c r="K10">
+        <v>6.3940593223914632</v>
+      </c>
+      <c r="L10">
+        <v>6.2283068224969425</v>
+      </c>
+      <c r="M10">
+        <v>6.0625543226024226</v>
+      </c>
+      <c r="N10">
+        <v>5.9754061010083985</v>
+      </c>
+      <c r="O10">
+        <v>5.8882578794143754</v>
+      </c>
+      <c r="P10">
+        <v>5.8216151217248244</v>
+      </c>
+      <c r="Q10">
+        <v>5.7549723640352735</v>
+      </c>
+      <c r="R10">
+        <v>5.4468208092485551</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>45</v>
+      </c>
+      <c r="B11">
+        <v>8.0114847474790061</v>
+      </c>
+      <c r="C11">
+        <v>7.8601999915615366</v>
+      </c>
+      <c r="D11">
+        <v>7.6619805071515952</v>
+      </c>
+      <c r="E11">
+        <v>7.4637610227416582</v>
+      </c>
+      <c r="F11">
+        <v>7.289464579553611</v>
+      </c>
+      <c r="G11">
+        <v>7.115168136365563</v>
+      </c>
+      <c r="H11">
+        <v>6.9955529302561157</v>
+      </c>
+      <c r="I11">
+        <v>6.8759377241466693</v>
+      </c>
+      <c r="J11">
+        <v>6.5820260748491659</v>
+      </c>
+      <c r="K11">
+        <v>6.2881144255516617</v>
+      </c>
+      <c r="L11">
+        <v>6.1684992194422152</v>
+      </c>
+      <c r="M11">
+        <v>6.0488840133327688</v>
+      </c>
+      <c r="N11">
+        <v>5.9942027762541672</v>
+      </c>
+      <c r="O11">
+        <v>5.9395215391755665</v>
+      </c>
+      <c r="P11">
+        <v>5.860917260875075</v>
+      </c>
+      <c r="Q11">
+        <v>5.7823129825745827</v>
+      </c>
+      <c r="R11">
+        <v>5.4162090809911625</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>50</v>
+      </c>
+      <c r="B12">
+        <v>7.8892493987595431</v>
+      </c>
+      <c r="C12">
+        <v>7.7405847854520893</v>
+      </c>
+      <c r="D12">
+        <v>7.5953377494620504</v>
+      </c>
+      <c r="E12">
+        <v>7.4500907134720133</v>
+      </c>
+      <c r="F12">
+        <v>7.2962997341884375</v>
+      </c>
+      <c r="G12">
+        <v>7.1425087549048634</v>
+      </c>
+      <c r="H12">
+        <v>7.0092232395257668</v>
+      </c>
+      <c r="I12">
+        <v>6.8759377241466693</v>
+      </c>
+      <c r="J12">
+        <v>6.6418336779038887</v>
+      </c>
+      <c r="K12">
+        <v>6.407729631661109</v>
+      </c>
+      <c r="L12">
+        <v>6.2812792709168388</v>
+      </c>
+      <c r="M12">
+        <v>6.1548289101725695</v>
+      </c>
+      <c r="N12">
+        <v>6.0078730855238218</v>
+      </c>
+      <c r="O12">
+        <v>5.860917260875075</v>
+      </c>
+      <c r="P12">
+        <v>5.8216151217248298</v>
+      </c>
+      <c r="Q12">
+        <v>5.7823129825745827</v>
+      </c>
+      <c r="R12">
+        <v>5.4615977626019445</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>55</v>
+      </c>
+      <c r="B13">
+        <v>7.7670140500400855</v>
+      </c>
+      <c r="C13">
+        <v>7.620969579342642</v>
+      </c>
+      <c r="D13">
+        <v>7.5286949917725048</v>
+      </c>
+      <c r="E13">
+        <v>7.4364204042023676</v>
+      </c>
+      <c r="F13">
+        <v>7.3031348888232657</v>
+      </c>
+      <c r="G13">
+        <v>7.1698493734441637</v>
+      </c>
+      <c r="H13">
+        <v>7.0228935487954169</v>
+      </c>
+      <c r="I13">
+        <v>6.8759377241466693</v>
+      </c>
+      <c r="J13">
+        <v>6.7016412809586123</v>
+      </c>
+      <c r="K13">
+        <v>6.5273448377705563</v>
+      </c>
+      <c r="L13">
+        <v>6.3940593223914632</v>
+      </c>
+      <c r="M13">
+        <v>6.2607738070123702</v>
+      </c>
+      <c r="N13">
+        <v>6.0215433947934764</v>
+      </c>
+      <c r="O13">
+        <v>5.7823129825745827</v>
+      </c>
+      <c r="P13">
+        <v>5.7823129825745827</v>
+      </c>
+      <c r="Q13">
+        <v>5.7823129825745827</v>
+      </c>
+      <c r="R13">
+        <v>5.5069864442127301</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>60</v>
+      </c>
+      <c r="B14">
+        <v>8.1611746339816964</v>
+      </c>
+      <c r="C14">
+        <v>8.0071558162102932</v>
+      </c>
+      <c r="D14">
+        <v>7.7679254039913985</v>
+      </c>
+      <c r="E14">
+        <v>7.5286949917725048</v>
+      </c>
+      <c r="F14">
+        <v>7.3082612547993797</v>
+      </c>
+      <c r="G14">
+        <v>7.0878275178262538</v>
+      </c>
+      <c r="H14">
+        <v>7.0553605333108358</v>
+      </c>
+      <c r="I14">
+        <v>7.0228935487954169</v>
+      </c>
+      <c r="J14">
+        <v>6.7887895025526364</v>
+      </c>
+      <c r="K14">
+        <v>6.5546854563098567</v>
+      </c>
+      <c r="L14">
+        <v>6.3615923378760399</v>
+      </c>
+      <c r="M14">
+        <v>6.1684992194422241</v>
+      </c>
+      <c r="N14">
+        <v>6.0147082401586491</v>
+      </c>
+      <c r="O14">
+        <v>5.860917260875075</v>
+      </c>
+      <c r="P14">
+        <v>5.8421205856293028</v>
+      </c>
+      <c r="Q14">
+        <v>5.8233239103835288</v>
+      </c>
+      <c r="R14">
+        <v>5.4613699241141145</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>65</v>
+      </c>
+      <c r="B15">
+        <v>8.5553352179233073</v>
+      </c>
+      <c r="C15">
+        <v>8.3933420530779426</v>
+      </c>
+      <c r="D15">
+        <v>8.0071558162102932</v>
+      </c>
+      <c r="E15">
+        <v>7.620969579342642</v>
+      </c>
+      <c r="F15">
+        <v>7.3133876207754938</v>
+      </c>
+      <c r="G15">
+        <v>7.0058056622083447</v>
+      </c>
+      <c r="H15">
+        <v>7.0878275178262538</v>
+      </c>
+      <c r="I15">
+        <v>7.1698493734441637</v>
+      </c>
+      <c r="J15">
+        <v>6.8759377241466613</v>
+      </c>
+      <c r="K15">
+        <v>6.582026074849157</v>
+      </c>
+      <c r="L15">
+        <v>6.3291253533606175</v>
+      </c>
+      <c r="M15">
+        <v>6.0762246318720772</v>
+      </c>
+      <c r="N15">
+        <v>6.0078730855238218</v>
+      </c>
+      <c r="O15">
+        <v>5.9395215391755665</v>
+      </c>
+      <c r="P15">
+        <v>5.9019281886840211</v>
+      </c>
+      <c r="Q15">
+        <v>5.8643348381924749</v>
+      </c>
+      <c r="R15">
+        <v>5.4157534040155006</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>70</v>
+      </c>
+      <c r="B16">
+        <v>8.9229526180330048</v>
+      </c>
+      <c r="C16">
+        <v>8.8478798362938402</v>
+      </c>
+      <c r="D16">
+        <v>8.2207543985485909</v>
+      </c>
+      <c r="E16">
+        <v>7.5936289608033398</v>
+      </c>
+      <c r="F16">
+        <v>7.3800303784650438</v>
+      </c>
+      <c r="G16">
+        <v>7.1664317961267461</v>
+      </c>
+      <c r="H16">
+        <v>7.120294502341677</v>
+      </c>
+      <c r="I16">
+        <v>7.074157208556608</v>
+      </c>
+      <c r="J16">
+        <v>6.8947343993924335</v>
+      </c>
+      <c r="K16">
+        <v>6.715311590228259</v>
+      </c>
+      <c r="L16">
+        <v>6.4419054048352402</v>
+      </c>
+      <c r="M16">
+        <v>6.1684992194422241</v>
+      </c>
+      <c r="N16">
+        <v>6.1138179823636181</v>
+      </c>
+      <c r="O16">
+        <v>6.0591367452850138</v>
+      </c>
+      <c r="P16">
+        <v>5.9736973123496906</v>
+      </c>
+      <c r="Q16">
+        <v>5.8882578794143665</v>
+      </c>
+      <c r="R16">
+        <v>5.4349569337038242</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>75</v>
+      </c>
+      <c r="B17">
+        <v>9.2905700181427022</v>
+      </c>
+      <c r="C17">
+        <v>9.3024176195097361</v>
+      </c>
+      <c r="D17">
+        <v>8.4343529808868887</v>
+      </c>
+      <c r="E17">
+        <v>7.5662883422640412</v>
+      </c>
+      <c r="F17">
+        <v>7.4466731361545948</v>
+      </c>
+      <c r="G17">
+        <v>7.3270579300451484</v>
+      </c>
+      <c r="H17">
+        <v>7.1527614868571003</v>
+      </c>
+      <c r="I17">
+        <v>6.9784650436690523</v>
+      </c>
+      <c r="J17">
+        <v>6.9135310746382057</v>
+      </c>
+      <c r="K17">
+        <v>6.84859710560736</v>
+      </c>
+      <c r="L17">
+        <v>6.5546854563098655</v>
+      </c>
+      <c r="M17">
+        <v>6.2607738070123702</v>
+      </c>
+      <c r="N17">
+        <v>6.2197628792034161</v>
+      </c>
+      <c r="O17">
+        <v>6.1787519513944611</v>
+      </c>
+      <c r="P17">
+        <v>6.0454664360153592</v>
+      </c>
+      <c r="Q17">
+        <v>5.9121809206362581</v>
+      </c>
+      <c r="R17">
+        <v>5.454160463392145</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>80</v>
+      </c>
+      <c r="B18">
+        <v>9.3502637019535157</v>
+      </c>
+      <c r="C18">
+        <v>9.1144508670520334</v>
+      </c>
+      <c r="D18">
+        <v>8.594979114805291</v>
+      </c>
+      <c r="E18">
+        <v>8.0755073625585485</v>
+      </c>
+      <c r="F18">
+        <v>7.7354584194759752</v>
+      </c>
+      <c r="G18">
+        <v>7.3954094763934037</v>
+      </c>
+      <c r="H18">
+        <v>7.260415172355601</v>
+      </c>
+      <c r="I18">
+        <v>7.1254208683178</v>
+      </c>
+      <c r="J18">
+        <v>7.0075144508670579</v>
+      </c>
+      <c r="K18">
+        <v>6.889608033416315</v>
+      </c>
+      <c r="L18">
+        <v>6.6691742964431953</v>
+      </c>
+      <c r="M18">
+        <v>6.4487405594700729</v>
+      </c>
+      <c r="N18">
+        <v>6.4145647862959407</v>
+      </c>
+      <c r="O18">
+        <v>6.3803890131218086</v>
+      </c>
+      <c r="P18">
+        <v>6.1872958946879892</v>
+      </c>
+      <c r="Q18">
+        <v>5.9942027762541672</v>
+      </c>
+      <c r="R18">
+        <v>5.601295303995613</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>85</v>
+      </c>
+      <c r="B19">
+        <v>9.4099573857643257</v>
+      </c>
+      <c r="C19">
+        <v>8.9264841145943308</v>
+      </c>
+      <c r="D19">
+        <v>8.7556052487236933</v>
+      </c>
+      <c r="E19">
+        <v>8.584726382853054</v>
+      </c>
+      <c r="F19">
+        <v>8.0242437027973548</v>
+      </c>
+      <c r="G19">
+        <v>7.4637610227416582</v>
+      </c>
+      <c r="H19">
+        <v>7.3680688578541034</v>
+      </c>
+      <c r="I19">
+        <v>7.2723766929665477</v>
+      </c>
+      <c r="J19">
+        <v>7.1014978270959084</v>
+      </c>
+      <c r="K19">
+        <v>6.93061896122527</v>
+      </c>
+      <c r="L19">
+        <v>6.7836631365765232</v>
+      </c>
+      <c r="M19">
+        <v>6.6367073119277755</v>
+      </c>
+      <c r="N19">
+        <v>6.6093666933884663</v>
+      </c>
+      <c r="O19">
+        <v>6.582026074849157</v>
+      </c>
+      <c r="P19">
+        <v>6.3291253533606175</v>
+      </c>
+      <c r="Q19">
+        <v>6.0762246318720772</v>
+      </c>
+      <c r="R19">
+        <v>5.7484301445990811</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>90</v>
+      </c>
+      <c r="B20">
+        <v>10.104978692882163</v>
+      </c>
+      <c r="C20">
+        <v>9.7159444749166788</v>
+      </c>
+      <c r="D20">
+        <v>9.1828024134002852</v>
+      </c>
+      <c r="E20">
+        <v>8.6496603518838917</v>
+      </c>
+      <c r="F20">
+        <v>8.1421501202480933</v>
+      </c>
+      <c r="G20">
+        <v>7.6346398886122966</v>
+      </c>
+      <c r="H20">
+        <v>7.4671786000590714</v>
+      </c>
+      <c r="I20">
+        <v>7.299717311505848</v>
+      </c>
+      <c r="J20">
+        <v>7.1749757394202813</v>
+      </c>
+      <c r="K20">
+        <v>7.0502341673347173</v>
+      </c>
+      <c r="L20">
+        <v>6.9357453272013876</v>
+      </c>
+      <c r="M20">
+        <v>6.8212564870680596</v>
+      </c>
+      <c r="N20">
+        <v>6.6879709716889586</v>
+      </c>
+      <c r="O20">
+        <v>6.5546854563098567</v>
+      </c>
+      <c r="P20">
+        <v>6.4213999409307636</v>
+      </c>
+      <c r="Q20">
+        <v>6.2881144255516705</v>
+      </c>
+      <c r="R20">
+        <v>5.7367941075421784</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>95</v>
+      </c>
+      <c r="B21">
+        <v>10.8</v>
+      </c>
+      <c r="C21">
+        <v>10.505404835239025</v>
+      </c>
+      <c r="D21">
+        <v>9.6099995780768772</v>
+      </c>
+      <c r="E21">
+        <v>8.7145943209147294</v>
+      </c>
+      <c r="F21">
+        <v>8.2600565376988335</v>
+      </c>
+      <c r="G21">
+        <v>7.8055187544829359</v>
+      </c>
+      <c r="H21">
+        <v>7.5662883422640412</v>
+      </c>
+      <c r="I21">
+        <v>7.3270579300451484</v>
+      </c>
+      <c r="J21">
+        <v>7.2484536517446561</v>
+      </c>
+      <c r="K21">
+        <v>7.1698493734441637</v>
+      </c>
+      <c r="L21">
+        <v>7.0878275178262538</v>
+      </c>
+      <c r="M21">
+        <v>7.0058056622083447</v>
+      </c>
+      <c r="N21">
+        <v>6.76657524998945</v>
+      </c>
+      <c r="O21">
+        <v>6.5273448377705563</v>
+      </c>
+      <c r="P21">
+        <v>6.5136745285009106</v>
+      </c>
+      <c r="Q21">
+        <v>6.5000042192312648</v>
+      </c>
+      <c r="R21">
+        <v>5.725158070485274</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>100</v>
+      </c>
+      <c r="B22">
+        <v>9.9554526902040603</v>
+      </c>
+      <c r="C22">
+        <v>9.6722954172486677</v>
+      </c>
+      <c r="D22">
+        <v>9.0522449641254354</v>
+      </c>
+      <c r="E22">
+        <v>8.432194511002205</v>
+      </c>
+      <c r="F22">
+        <v>7.9934255494438418</v>
+      </c>
+      <c r="G22">
+        <v>7.5546565878854803</v>
+      </c>
+      <c r="H22">
+        <v>7.4739537971971011</v>
+      </c>
+      <c r="I22">
+        <v>7.3932510065087245</v>
+      </c>
+      <c r="J22">
+        <v>7.201596867998024</v>
+      </c>
+      <c r="K22">
+        <v>7.0099427294873182</v>
+      </c>
+      <c r="L22">
+        <v>6.8270423855089426</v>
+      </c>
+      <c r="M22">
+        <v>6.6441420415305643</v>
+      </c>
+      <c r="N22">
+        <v>6.5119357610938042</v>
+      </c>
+      <c r="O22">
+        <v>6.379729480657045</v>
+      </c>
+      <c r="P22">
+        <v>6.267489046653596</v>
+      </c>
+      <c r="Q22">
+        <v>6.1552486126501451</v>
+      </c>
+      <c r="R22">
+        <v>5.6019959501724648</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6053,7 +8091,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C196"/>
   <sheetFormatPr defaultColWidth="23.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6979,7 +9017,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:BT193"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -19256,7 +21294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B197"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -20069,7 +22107,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -20655,7 +22693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:BT196"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -41151,7 +43189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:A192"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -41827,802 +43865,4 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:B193"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B23">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>28</v>
-      </c>
-      <c r="B29">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>29</v>
-      </c>
-      <c r="B30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>31</v>
-      </c>
-      <c r="B32">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>32</v>
-      </c>
-      <c r="B33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>33</v>
-      </c>
-      <c r="B34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>36</v>
-      </c>
-      <c r="B37">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>37</v>
-      </c>
-      <c r="B38">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>38</v>
-      </c>
-      <c r="B39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>39</v>
-      </c>
-      <c r="B40">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>40</v>
-      </c>
-      <c r="B41">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="1"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="1"/>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="1"/>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="1"/>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="1"/>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="1"/>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="1"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" s="1"/>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" s="1"/>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" s="1"/>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" s="1"/>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" s="1"/>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" s="1"/>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" s="1"/>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" s="1"/>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" s="1"/>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" s="1"/>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" s="1"/>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" s="1"/>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" s="1"/>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" s="1"/>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" s="1"/>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" s="1"/>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" s="1"/>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" s="1"/>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" s="1"/>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" s="1"/>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" s="1"/>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" s="1"/>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71" s="1"/>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" s="1"/>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" s="1"/>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" s="1"/>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" s="1"/>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" s="1"/>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" s="1"/>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" s="1"/>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" s="1"/>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80" s="1"/>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" s="1"/>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" s="1"/>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" s="1"/>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" s="1"/>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85" s="1"/>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" s="1"/>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" s="1"/>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" s="1"/>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" s="1"/>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" s="1"/>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" s="1"/>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" s="1"/>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" s="1"/>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" s="1"/>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" s="1"/>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" s="1"/>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97" s="1"/>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98" s="1"/>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A99" s="1"/>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100" s="1"/>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A101" s="1"/>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A102" s="1"/>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A103" s="1"/>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A104" s="1"/>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A105" s="1"/>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A106" s="1"/>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A107" s="1"/>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A108" s="1"/>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A109" s="1"/>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A110" s="1"/>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A111" s="1"/>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A112" s="1"/>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A113" s="1"/>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A114" s="1"/>
-    </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A115" s="1"/>
-    </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A116" s="1"/>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A117" s="1"/>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A118" s="1"/>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A119" s="1"/>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A120" s="1"/>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A121" s="1"/>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A122" s="1"/>
-    </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A123" s="1"/>
-    </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A124" s="1"/>
-    </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A125" s="1"/>
-    </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A126" s="1"/>
-    </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A127" s="1"/>
-    </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A128" s="1"/>
-    </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A129" s="1"/>
-    </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A130" s="1"/>
-    </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A131" s="1"/>
-    </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A132" s="1"/>
-    </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A133" s="1"/>
-    </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A134" s="1"/>
-    </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A135" s="1"/>
-    </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A136" s="1"/>
-    </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A137" s="1"/>
-    </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A138" s="1"/>
-    </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A139" s="1"/>
-    </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A140" s="1"/>
-    </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A141" s="1"/>
-    </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A142" s="1"/>
-    </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A143" s="1"/>
-    </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A144" s="1"/>
-    </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A145" s="1"/>
-    </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A146" s="1"/>
-    </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A147" s="1"/>
-    </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A148" s="1"/>
-    </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A149" s="1"/>
-    </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A150" s="1"/>
-    </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A151" s="1"/>
-    </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A152" s="1"/>
-    </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A153" s="1"/>
-    </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A154" s="1"/>
-    </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A155" s="1"/>
-    </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A156" s="1"/>
-    </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A157" s="1"/>
-    </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A158" s="1"/>
-    </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A159" s="1"/>
-    </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A160" s="1"/>
-    </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A161" s="1"/>
-    </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A162" s="1"/>
-    </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A163" s="1"/>
-    </row>
-    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A164" s="1"/>
-    </row>
-    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A165" s="1"/>
-    </row>
-    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A166" s="1"/>
-    </row>
-    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A167" s="1"/>
-    </row>
-    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A168" s="1"/>
-    </row>
-    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A169" s="1"/>
-    </row>
-    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A170" s="1"/>
-    </row>
-    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A171" s="1"/>
-    </row>
-    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A172" s="1"/>
-    </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A173" s="1"/>
-    </row>
-    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A174" s="1"/>
-    </row>
-    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A175" s="1"/>
-    </row>
-    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A176" s="1"/>
-    </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A177" s="1"/>
-    </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A178" s="1"/>
-    </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A179" s="1"/>
-    </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A180" s="1"/>
-    </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A181" s="1"/>
-    </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A182" s="1"/>
-    </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A183" s="1"/>
-    </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A184" s="1"/>
-    </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A185" s="1"/>
-    </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A186" s="1"/>
-    </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A187" s="1"/>
-    </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A188" s="1"/>
-    </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A189" s="1"/>
-    </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A190" s="1"/>
-    </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A191" s="1"/>
-    </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A192" s="1"/>
-    </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A193" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>